<commit_message>
:wrench: Configuration files and Browser config form is updated to separate Organization creation and references
</commit_message>
<xml_diff>
--- a/src/main/resources/config.xlsx
+++ b/src/main/resources/config.xlsx
@@ -35,6 +35,7 @@
     <sheet name="Dataset Types" sheetId="18" state="hidden" r:id="rId20"/>
     <sheet name="Countries" sheetId="19" state="hidden" r:id="rId21"/>
     <sheet name="Value Sets" sheetId="15" state="hidden" r:id="rId22"/>
+    <sheet name="Organizations" sheetId="32" r:id="rId34"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">Catalog!$A$1:$H$28</definedName>
@@ -57536,6 +57537,11 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="22.5" customHeight="1">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGE</t>
+        </is>
+      </c>
       <c r="A7" s="59" t="s">
         <v>2444</v>
       </c>
@@ -57551,15 +57557,14 @@
       <c r="E7" s="8" t="s">
         <v>2448</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>2428</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQUIRED - Organization ID</t>
+        </is>
       </c>
       <c r="G7" s="14" t="str">
         <f t="shared" si="0"/>
         <v>STAGE</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>2426</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="22.5" customHeight="1">
@@ -57570,14 +57575,15 @@
       <c r="E8" s="8" t="s">
         <v>2449</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>2446</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G8" s="14" t="str">
         <f>_xlfn.IFNA(INDEX(Corporate_Bodies[Uri], MATCH(H8, Corporate_Bodies[Label], 0)),"")</f>
         <v/>
       </c>
-      <c r="H8" s="8"/>
     </row>
     <row r="9" spans="1:26" ht="38.25" customHeight="1">
       <c r="A9" s="45" t="s">
@@ -57782,6 +57788,11 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="26.25" customHeight="1">
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGE</t>
+        </is>
+      </c>
       <c r="A17" s="56" t="s">
         <v>2434</v>
       </c>
@@ -57797,13 +57808,14 @@
       <c r="E17" s="8" t="s">
         <v>2448</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>2428</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQUIRED - Organization ID</t>
+        </is>
       </c>
       <c r="G17" s="47" t="s">
         <v>2426</v>
       </c>
-      <c r="H17" s="46"/>
     </row>
     <row r="18" spans="1:8" s="5" customFormat="1" ht="26.25" customHeight="1">
       <c r="A18" s="56"/>
@@ -57813,15 +57825,14 @@
       <c r="E18" s="8" t="s">
         <v>2476</v>
       </c>
-      <c r="F18" s="13" t="s">
-        <v>2432</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G18" s="14" t="str">
         <f t="shared" ref="G18:G26" si="1">IF(H18="","",H18)</f>
         <v>https://stage-healthyageing.eu/contact</v>
-      </c>
-      <c r="H18" s="48" t="s">
-        <v>2477</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="5" customFormat="1" ht="26.25" customHeight="1">
@@ -57832,15 +57843,14 @@
       <c r="E19" s="8" t="s">
         <v>2478</v>
       </c>
-      <c r="F19" s="13" t="s">
-        <v>2432</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G19" s="14" t="str">
         <f t="shared" si="1"/>
         <v>sylvain.sebert@oulu.fi</v>
-      </c>
-      <c r="H19" s="48" t="s">
-        <v>2479</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="5" customFormat="1" ht="26.25" customHeight="1">
@@ -57851,14 +57861,15 @@
       <c r="E20" s="8" t="s">
         <v>2449</v>
       </c>
-      <c r="F20" s="8" t="s">
-        <v>2446</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G20" s="14" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="H20" s="8"/>
     </row>
     <row r="21" spans="1:8" s="5" customFormat="1" ht="48" customHeight="1">
       <c r="A21" s="56"/>
@@ -57868,15 +57879,14 @@
       <c r="E21" s="8" t="s">
         <v>2480</v>
       </c>
-      <c r="F21" s="8" t="s">
-        <v>2446</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G21" s="14" t="str">
         <f t="shared" si="1"/>
         <v xml:space="preserve">The catalog is maintained and published by the STAGE consortium </v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>2481</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="5" customFormat="1" ht="30.75" customHeight="1">
@@ -57887,15 +57897,14 @@
       <c r="E22" s="13" t="s">
         <v>2482</v>
       </c>
-      <c r="F22" s="8" t="s">
-        <v>2446</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G22" s="14" t="str">
         <f t="shared" si="1"/>
         <v>true</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>2483</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="33" customHeight="1">
@@ -58055,8 +58064,6 @@
     <hyperlink ref="C28" r:id="rId4" location="Catalogue" display="https://healthdataeu.pages.code.europa.eu/healthdcat-ap/releases/release-5/ - Catalogue" xr:uid="{44F128B9-B51C-494F-8B1B-D19E5997EFBB}"/>
     <hyperlink ref="H12" r:id="rId5" xr:uid="{9CE524A8-D6A9-4F13-BC70-92E587998D83}"/>
     <hyperlink ref="H14" r:id="rId6" xr:uid="{532E2CA4-B4B3-44B6-A9EC-D832A6DFCEDE}"/>
-    <hyperlink ref="H19" r:id="rId7" xr:uid="{0CDCFC7B-DEE2-40EE-9456-A4CB64D52EA6}"/>
-    <hyperlink ref="H18" r:id="rId8" xr:uid="{00B0F471-AF39-4338-9B64-AD76DAB0FEB4}"/>
     <hyperlink ref="C25" r:id="rId9" location="Catalogue" display="https://healthdataeu.pages.code.europa.eu/healthdcat-ap/releases/release-5/ - Catalogue" xr:uid="{E249F9AD-4D7A-4D66-A5AE-A4C3375233D2}"/>
     <hyperlink ref="C26" r:id="rId10" location="Catalogue" display="https://healthdataeu.pages.code.europa.eu/healthdcat-ap/releases/release-5/ - Catalogue" xr:uid="{797442FA-FF85-4C42-992D-15B8BDA31E1F}"/>
   </hyperlinks>
@@ -64747,6 +64754,172 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="46" customWidth="1"/>
+    <col min="5" max="7" width="34" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
+    <col min="9" max="10" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organization ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canonical IRI</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contact Page</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contact Email</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Homepage</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trusted Data Holder</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Other Identifiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://stage-healthyageing.eu/contact</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sylvain.sebert@oulu.fi</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The catalog is maintained and published by the STAGE consortium</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OULU</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OULU</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">http://publications.europa.eu/resource/authority/corporate-body/EUI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://oulu.fi</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">info@oulu.edu.fi</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The publisher provides this dataset metadata without warranties of any kind. The publisher shall not be liable for any use of the data beyond the conditions defined by the applicable access and reuse policies.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JOHN_DOE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">John Doe</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">john.doe@oulu.fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JANE_DOE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jane Doe</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E326DCC6-C92E-4984-B17B-69868B6CF2DC}">
   <dimension ref="A1:B4"/>
@@ -67741,6 +67914,11 @@
       </c>
     </row>
     <row r="11" spans="1:9" s="5" customFormat="1" ht="29.65" customHeight="1">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OULU</t>
+        </is>
+      </c>
       <c r="A11" s="56" t="s">
         <v>3160</v>
       </c>
@@ -67756,15 +67934,14 @@
       <c r="E11" s="5" t="s">
         <v>2448</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>2428</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQUIRED - Organization ID</t>
+        </is>
       </c>
       <c r="G11" s="36" t="str">
         <f>H11</f>
         <v>OULU</v>
-      </c>
-      <c r="H11" t="s">
-        <v>3172</v>
       </c>
     </row>
     <row r="12" spans="1:9" s="5" customFormat="1" ht="24.4" customHeight="1">
@@ -67775,15 +67952,14 @@
       <c r="E12" s="5" t="s">
         <v>2449</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>2446</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G12" s="34" t="str">
         <f>_xlfn.IFNA(INDEX(Corporate_Bodies[Uri], MATCH(H12, Corporate_Bodies[Label], 0)),"")</f>
         <v>http://publications.europa.eu/resource/authority/corporate-body/EUI</v>
-      </c>
-      <c r="H12" t="s">
-        <v>3173</v>
       </c>
     </row>
     <row r="13" spans="1:9" s="5" customFormat="1" ht="25.9" customHeight="1">
@@ -67794,15 +67970,14 @@
       <c r="E13" s="5" t="s">
         <v>3174</v>
       </c>
-      <c r="F13" s="15" t="s">
-        <v>2432</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G13" s="36" t="str">
         <f>IF(H13="","",H13)</f>
         <v>https://oulu.fi</v>
-      </c>
-      <c r="H13" s="16" t="s">
-        <v>3175</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="5" customFormat="1" ht="27" customHeight="1">
@@ -67813,18 +67988,22 @@
       <c r="E14" s="5" t="s">
         <v>3176</v>
       </c>
-      <c r="F14" s="15" t="s">
-        <v>2432</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G14" s="36" t="str">
         <f>IF(H14="","",H14)</f>
         <v>info@oulu.edu.fi</v>
       </c>
-      <c r="H14" s="16" t="s">
-        <v>3177</v>
-      </c>
     </row>
     <row r="15" spans="1:9" ht="29.65" customHeight="1">
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OULU</t>
+        </is>
+      </c>
       <c r="A15" s="60" t="s">
         <v>2426</v>
       </c>
@@ -67840,15 +68019,14 @@
       <c r="E15" t="s">
         <v>2448</v>
       </c>
-      <c r="F15" t="s">
-        <v>2428</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQUIRED - Organization ID</t>
+        </is>
       </c>
       <c r="G15" s="34" t="str">
         <f>IF(H15="","",H15)</f>
         <v>OULU</v>
-      </c>
-      <c r="H15" t="s">
-        <v>3172</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="25.9" customHeight="1">
@@ -67859,15 +68037,14 @@
       <c r="E16" t="s">
         <v>2476</v>
       </c>
-      <c r="F16" s="28" t="s">
-        <v>2432</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G16" s="34" t="str">
         <f t="shared" ref="G16:G17" si="0">IF(H16="","",H16)</f>
         <v>https://oulu.fi</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>3175</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="30" customHeight="1">
@@ -67878,15 +68055,14 @@
       <c r="E17" t="s">
         <v>2478</v>
       </c>
-      <c r="F17" s="28" t="s">
-        <v>2432</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G17" s="34" t="str">
         <f t="shared" si="0"/>
         <v>info@oulu.edu.fi</v>
-      </c>
-      <c r="H17" s="16" t="s">
-        <v>3177</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="30.4" customHeight="1">
@@ -67897,15 +68073,14 @@
       <c r="E18" t="s">
         <v>2449</v>
       </c>
-      <c r="F18" t="s">
-        <v>2446</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G18" s="34" t="str">
         <f>_xlfn.IFNA(INDEX(Corporate_Bodies[Uri], MATCH(H18, Corporate_Bodies[Label], 0)),"")</f>
         <v>http://publications.europa.eu/resource/authority/corporate-body/EUI</v>
-      </c>
-      <c r="H18" t="s">
-        <v>3173</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="84.4" customHeight="1">
@@ -67916,15 +68091,14 @@
       <c r="E19" t="s">
         <v>3179</v>
       </c>
-      <c r="F19" t="s">
-        <v>2446</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G19" s="34" t="str">
         <f>IF(H19="","",H19)</f>
         <v>The publisher provides this dataset metadata without warranties of any kind. The publisher shall not be liable for any use of the data beyond the conditions defined by the applicable access and reuse policies.</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>3180</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="25.15" customHeight="1">
@@ -67935,16 +68109,15 @@
       <c r="E20" s="28" t="s">
         <v>2482</v>
       </c>
-      <c r="F20" t="s">
-        <v>2446</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G20" s="34" t="str">
         <f>IF(H20="","",H20)</f>
         <v>true</v>
       </c>
-      <c r="H20" t="s">
-        <v>2483</v>
-      </c>
     </row>
     <row r="21" spans="1:16" ht="25.5" customHeight="1">
       <c r="A21" s="17" t="s">
@@ -68188,6 +68361,11 @@
       <c r="I28" s="29"/>
     </row>
     <row r="29" spans="1:16" ht="29.65" customHeight="1">
+      <c r="H29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JOHN_DOE</t>
+        </is>
+      </c>
       <c r="A29" s="59" t="s">
         <v>2444</v>
       </c>
@@ -68203,15 +68381,14 @@
       <c r="E29" t="s">
         <v>2448</v>
       </c>
-      <c r="F29" t="s">
-        <v>2428</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQUIRED - Organization ID</t>
+        </is>
       </c>
       <c r="G29" s="34" t="str">
         <f>IF(H29="","",H29)</f>
         <v>John Doe</v>
-      </c>
-      <c r="H29" t="s">
-        <v>3208</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="31.15" customHeight="1">
@@ -68222,15 +68399,14 @@
       <c r="E30" t="s">
         <v>2449</v>
       </c>
-      <c r="F30" t="s">
-        <v>2446</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FROM Organizations sheet</t>
+        </is>
       </c>
       <c r="G30" s="34" t="str">
         <f t="shared" ref="G30:G39" si="1">IF(H30="","",H30)</f>
         <v>john.doe@oulu.fi</v>
-      </c>
-      <c r="H30" s="16" t="s">
-        <v>3169</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="27.4" customHeight="1">
@@ -68918,6 +69094,11 @@
       </c>
     </row>
     <row r="58" spans="1:10" ht="25.5" customHeight="1">
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JANE_DOE</t>
+        </is>
+      </c>
       <c r="A58" s="59" t="s">
         <v>2444</v>
       </c>
@@ -68933,15 +69114,14 @@
       <c r="E58" t="s">
         <v>2448</v>
       </c>
-      <c r="F58" t="s">
-        <v>2428</v>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQUIRED - Organization ID</t>
+        </is>
       </c>
       <c r="G58" s="34" t="str">
         <f>_xlfn.TEXTJOIN(",",FALSE,H58:Z58)</f>
         <v>Jane Doe,,,,,,,,,,,,,,,,,,</v>
-      </c>
-      <c r="H58" t="s">
-        <v>3269</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="23.65" customHeight="1">
@@ -69372,19 +69552,14 @@
     <hyperlink ref="H45" r:id="rId8" xr:uid="{22C4E91C-80E4-4341-AF22-087992F26B4F}"/>
     <hyperlink ref="I45" r:id="rId9" xr:uid="{922F0CEE-D5E6-4213-BB08-60E19519CC4F}"/>
     <hyperlink ref="H9" r:id="rId10" xr:uid="{4672466C-1C4D-4A40-BB41-2EFEB59DC0D7}"/>
-    <hyperlink ref="H13" r:id="rId11" xr:uid="{2F597C57-8726-4B62-B478-C4986D05D8C8}"/>
-    <hyperlink ref="H14" r:id="rId12" xr:uid="{C2086C7D-0165-4A21-88B1-B2ED144D448E}"/>
     <hyperlink ref="H28" r:id="rId13" xr:uid="{D3D7D405-FAF2-4E8D-BDE2-068A7D230232}"/>
-    <hyperlink ref="H30" r:id="rId14" xr:uid="{E12FAF52-858B-47B1-BE4B-AEF123C32CC9}"/>
     <hyperlink ref="H31" r:id="rId15" xr:uid="{C63E20A4-16D7-401B-8E8C-C9983B29A6F9}"/>
     <hyperlink ref="H33" r:id="rId16" xr:uid="{56375A8F-31F1-4A83-B6B6-259E28A4763B}"/>
     <hyperlink ref="H34" r:id="rId17" xr:uid="{7AEDC613-AB16-4280-ABFE-C060E6BA2BA0}"/>
     <hyperlink ref="H37" r:id="rId18" xr:uid="{908048EB-1C26-4735-9EAB-AF7273605690}"/>
     <hyperlink ref="H38" r:id="rId19" xr:uid="{5C9FB907-6BE2-4BBD-B2AC-FA5DB06AE827}"/>
-    <hyperlink ref="H17" r:id="rId20" xr:uid="{6BC9FDEF-5BBC-45EC-AD83-E104D62CDF0A}"/>
     <hyperlink ref="H53" r:id="rId21" xr:uid="{AA48F2B6-1E4A-4025-8E44-127A0F3E8E37}"/>
     <hyperlink ref="H57" r:id="rId22" xr:uid="{AACCF0FD-4B7E-48AA-9CFB-7988FA4B403A}"/>
-    <hyperlink ref="H16" r:id="rId23" xr:uid="{27F937F0-0DA4-4A01-9CEF-BDFF0D07C378}"/>
     <hyperlink ref="H42" r:id="rId24" xr:uid="{BFD983AB-C524-4A71-8594-585520133497}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
:bug: R7 migration from explicit IP host to hdeu-dcat..., alongside a few config changes
</commit_message>
<xml_diff>
--- a/src/main/resources/config.xlsx
+++ b/src/main/resources/config.xlsx
@@ -9499,205 +9499,205 @@
     <t>party who has an interest in the resource or the use of the resource</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/ADMISSION_DISCHARGE</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/ADMISSION_DISCHARGE</t>
   </si>
   <si>
     <t>Admission Discharge</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/HOSPITAL_RECORDS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/HOSPITAL_RECORDS</t>
   </si>
   <si>
     <t>Hospital Records</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/HEALTHCARE_VISIT</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/HEALTHCARE_VISIT</t>
   </si>
   <si>
     <t>Healthcare Visit</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/OBSERVATIONAL_DATA</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/OBSERVATIONAL_DATA</t>
   </si>
   <si>
     <t>Observational Data</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/HEALTH_SURVEY</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/HEALTH_SURVEY</t>
   </si>
   <si>
     <t>Health Survey</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/SURVEILLANCE</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/SURVEILLANCE</t>
   </si>
   <si>
     <t>Surveillance</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/NONMEDICAL_APPLICATION</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/NONMEDICAL_APPLICATION</t>
   </si>
   <si>
     <t>Nonmedical Application</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/SAMPLE_COLLECTIONS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/SAMPLE_COLLECTIONS</t>
   </si>
   <si>
     <t>Sample Collections</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/QUALITY_REGISTRIES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/QUALITY_REGISTRIES</t>
   </si>
   <si>
     <t>Quality Registries</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/EHEALTH_APPLICATION</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/EHEALTH_APPLICATION</t>
   </si>
   <si>
     <t>Ehealth Application</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/ROUTINE_RECORDS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/ROUTINE_RECORDS</t>
   </si>
   <si>
     <t>Routine Records</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/HEALTH_REGISTRIES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/HEALTH_REGISTRIES</t>
   </si>
   <si>
     <t>Health Registries</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/RESEARCH_DATABASE</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/RESEARCH_DATABASE</t>
   </si>
   <si>
     <t>Research Database</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/RESEARCH_PROJECT</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/RESEARCH_PROJECT</t>
   </si>
   <si>
     <t>Research Project</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/MUNICIPAL_REPOSITORY</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/MUNICIPAL_REPOSITORY</t>
   </si>
   <si>
     <t>Municipal Repository</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/COHORT</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/COHORT</t>
   </si>
   <si>
     <t>Cohort</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/GEOSPATIAL_MONITORING</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/GEOSPATIAL_MONITORING</t>
   </si>
   <si>
     <t>Geospatial Monitoring</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/MODELS_SIMULATIONS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/MODELS_SIMULATIONS</t>
   </si>
   <si>
     <t>Models Simulations</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/CLINICAL_TRIAL</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/CLINICAL_TRIAL</t>
   </si>
   <si>
     <t>Clinical Trial</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/QUALITY_REGISTRY</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/QUALITY_REGISTRY</t>
   </si>
   <si>
     <t>Quality Registry</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/MEDICAL_REGISTRY</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/MEDICAL_REGISTRY</t>
   </si>
   <si>
     <t>Medical Registry</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/ADMINISTRATIVE_PROCESSES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/ADMINISTRATIVE_PROCESSES</t>
   </si>
   <si>
     <t>Administrative Processes</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/DISEASE_MONITORING</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/DISEASE_MONITORING</t>
   </si>
   <si>
     <t>Disease Monitoring</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/PRESCRIBING_DISPENSING</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/PRESCRIBING_DISPENSING</t>
   </si>
   <si>
     <t>Prescribing Dispensing</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/AUTOMATIC_GENERATION</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/AUTOMATIC_GENERATION</t>
   </si>
   <si>
     <t>Automatic Generation</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/LABORATORY_TESTS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/LABORATORY_TESTS</t>
   </si>
   <si>
     <t>Laboratory Tests</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/PROBABILITY_SURVEY</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/PROBABILITY_SURVEY</t>
   </si>
   <si>
     <t>Probability Survey</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/BIOBANK_COLLECTION</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/BIOBANK_COLLECTION</t>
   </si>
   <si>
     <t>Biobank Collection</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/MEASUREMENTS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/MEASUREMENTS</t>
   </si>
   <si>
     <t>Measurements</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/PATIENT_OUTCOMES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/PATIENT_OUTCOMES</t>
   </si>
   <si>
     <t>Patient Outcomes</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/CENSUS_DATA</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/CENSUS_DATA</t>
   </si>
   <si>
     <t>Census Data</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/MEDICAL_DEVICES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/MEDICAL_DEVICES</t>
   </si>
   <si>
     <t>Medical Devices</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/HEALTH_SURVEILLANCE</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/HEALTH_SURVEILLANCE</t>
   </si>
   <si>
     <t>Health Surveillance</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-activity/INSURANCE_CLAIMS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/INSURANCE_CLAIMS</t>
   </si>
   <si>
     <t>Insurance Claims</t>
@@ -23531,217 +23531,217 @@
     <t>Youth Working Party</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/ENVIRONMENTAL_HEALTH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/ENVIRONMENTAL_HEALTH</t>
   </si>
   <si>
     <t>Environmental, occupational radiation health (incl. WASH urban)</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/NUTRITION_SECURITY</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/NUTRITION_SECURITY</t>
   </si>
   <si>
     <t>Nutrition food security</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/TROPICAL_DISEASES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/TROPICAL_DISEASES</t>
   </si>
   <si>
     <t>Neglected tropical, parasitic fungal skin diseases</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/RESPIRATORY_DISEASES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/RESPIRATORY_DISEASES</t>
   </si>
   <si>
     <t>Respiratory infectious diseases</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/VECTOR_DISEASES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/VECTOR_DISEASES</t>
   </si>
   <si>
     <t>Vector-borne zoonotic viral diseases</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/EMERGENCY_SETTINGS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/EMERGENCY_SETTINGS</t>
   </si>
   <si>
     <t>Emergencies, disasters, travel humanitarian settings</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/REPRODUCTIVE_HEALTH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/REPRODUCTIVE_HEALTH</t>
   </si>
   <si>
     <t>Sexual reproductive health and rights</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/BLOOD_INFECTIONS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/BLOOD_INFECTIONS</t>
   </si>
   <si>
     <t>Blood-borne sexually transmitted infections</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/HEALTH_PRODUCTS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/HEALTH_PRODUCTS</t>
   </si>
   <si>
     <t>Health products, technologies, data research</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/LIFECOURSE_HEALTH</t>
-  </si>
-  <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/ENTERIC_INFECTIONS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/LIFECOURSE_HEALTH</t>
+  </si>
+  <si>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/ENTERIC_INFECTIONS</t>
   </si>
   <si>
     <t>Enteric, water- food-borne infections</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/NONCOMMUNICABLE_DISEASES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/NONCOMMUNICABLE_DISEASES</t>
   </si>
   <si>
     <t>Noncommunicable diseases ? metabolic cardiopulmonary</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/HEALTH_SYSTEMS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/HEALTH_SYSTEMS</t>
   </si>
   <si>
     <t>Health systems, quality, care models determinants</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/CLIMATE_HEALTH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/CLIMATE_HEALTH</t>
   </si>
   <si>
     <t>Climate planetary health</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/ANTIMICROBIAL_CONTROL</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/ANTIMICROBIAL_CONTROL</t>
   </si>
   <si>
     <t>Antimicrobial resistance infection control</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/MENTAL_HEALTH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/MENTAL_HEALTH</t>
   </si>
   <si>
     <t>Mental, neurological substance use</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/SENSORY_HEALTH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/SENSORY_HEALTH</t>
   </si>
   <si>
     <t>Oral, eye sensory health</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/IMMUNIZATION_DISEASES</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/IMMUNIZATION_DISEASES</t>
   </si>
   <si>
     <t>Immunization vaccine-preventable diseases</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/INJURY_PREVENTION</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/INJURY_PREVENTION</t>
   </si>
   <si>
     <t>Injuries, envenoming drowning</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/health-theme/CANCER_DISEASE</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/CANCER_DISEASE</t>
   </si>
   <si>
     <t>Cancer</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/PGEH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/PGEH</t>
   </si>
   <si>
     <t>Personal electronic health data automatically generated through medical devices</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/RQSH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/RQSH</t>
   </si>
   <si>
     <t>Data from research cohorts, questionnaires and surveys related to health, after the first publication of the related results</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/NRPE</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/NRPE</t>
   </si>
   <si>
     <t>Aggregated data on healthcare needs, resources allocated to healthcare, the provision of and access to healthcare, healthcare expenditure and financing</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/RMMD</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/RMMD</t>
   </si>
   <si>
     <t>Data from registries for medicinal products and medical devices</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/DIOH</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/DIOH</t>
   </si>
   <si>
     <t>Data on factors impacting on health, including socio-economic, environmental and behavioural determinants of health</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/EMRD</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/EMRD</t>
   </si>
   <si>
     <t>Other health data from medical devices</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/EHCT</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/EHCT</t>
   </si>
   <si>
     <t>Data from clinical trials, clinical studies, clinical investigations and performance studies subject to Regulation (EU) No 536/2014, Regulation (EU) 2024/1938 of the European Parliament and of the Council34, Regulation (EU) 2017/745 and Regulation (EU) 2017/746</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/EHRS</t>
-  </si>
-  <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/MRMR</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/EHRS</t>
+  </si>
+  <si>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/MRMR</t>
   </si>
   <si>
     <t>Data from medical registries and mortality registries</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/HRAD</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/HRAD</t>
   </si>
   <si>
     <t>Healthcare-related administrative data, including on dispensations, reimbursement claims and reimbursements</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/IDHP</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/IDHP</t>
   </si>
   <si>
     <t>Data on professional status, and on the specialisation and institution of health professionals involved in the treatment of a natural person</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/HGPD</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/HGPD</t>
   </si>
   <si>
     <t>Human genetic, epigenomic and genomic data</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/RPDG</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/RPDG</t>
   </si>
   <si>
     <t>Data on pathogens that impact human health</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/PHDR</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/PHDR</t>
   </si>
   <si>
     <t>Data from population-based health data registries such as public health registries</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/EINS</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/EINS</t>
   </si>
   <si>
     <t>Health data from biobanks and associated databases</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/HPML</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/HPML</t>
   </si>
   <si>
     <t>Other human molecular data such as proteomic, transcriptomic, metabolomic, lipidomic and other omic data</t>
   </si>
   <si>
-    <t>http://13.81.34.152:1101/resource/authority/healthcategories/WELA</t>
+    <t>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/WELA</t>
   </si>
   <si>
     <t>Data from wellness applications</t>
@@ -67631,7 +67631,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B89FB9D3-3C26-4805-A4F2-39333E3C7845}">
-  <dimension ref="A1:P75"/>
+  <dimension ref="A1:P76"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="17.42578125" customWidth="1"/>
@@ -68218,7 +68218,7 @@
       </c>
       <c r="G23" s="34" t="str">
         <f>INDEX(Health_Categories[Uri], MATCH(H23, Health_Categories[Label], 0))</f>
-        <v>http://13.81.34.152:1101/resource/authority/healthcategories/EHRS</v>
+        <v>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/healthcategories/EHRS</v>
       </c>
       <c r="H23" t="s">
         <v>3195</v>
@@ -68326,7 +68326,7 @@
       </c>
       <c r="G27" s="34" t="str">
         <f>INDEX(Health_Themes[Uri], MATCH(H27, Health_Themes[Label], 0))</f>
-        <v>http://13.81.34.152:1101/resource/authority/health-theme/LIFECOURSE_HEALTH</v>
+        <v>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-theme/LIFECOURSE_HEALTH</v>
       </c>
       <c r="H27" t="s">
         <v>3203</v>
@@ -69285,7 +69285,7 @@
       </c>
       <c r="G65" s="34" t="str" cm="1">
         <f t="array" aca="1" ref="G65" ca="1">INDIRECT("Helpers!A1")</f>
-        <v>http://13.81.34.152:1101/resource/authority/health-activity/EHEALTH_APPLICATION,http://13.81.34.152:1101/resource/authority/health-activity/OBSERVATIONAL_DATA,http://13.81.34.152:1101/resource/authority/health-activity/SURVEILLANCE</v>
+        <v>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/EHEALTH_APPLICATION,https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/OBSERVATIONAL_DATA,https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/SURVEILLANCE</v>
       </c>
       <c r="H65" t="s">
         <v>3093</v>
@@ -69445,6 +69445,43 @@
     <row r="75" spans="1:10">
       <c r="B75" s="41"/>
       <c r="E75" s="1"/>
+    </row>
+    <row r="76">
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Release 7. Whether the dataset holds structured data that can be described variable by variable. Leave empty to derive it: true when a data dictionary / extracted columns exist. When true, the CSVW variables description is mandatory.</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQUIRED</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">structured data</t>
+        </is>
+      </c>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEALTHDCAT-AP</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H26" xr:uid="{B89FB9D3-3C26-4805-A4F2-39333E3C7845}"/>
@@ -69582,19 +69619,19 @@
     <row r="1" spans="1:27">
       <c r="A1" t="str">
         <f>_xlfn.TEXTJOIN(",", TRUE, H1:AA1)</f>
-        <v>http://13.81.34.152:1101/resource/authority/health-activity/EHEALTH_APPLICATION,http://13.81.34.152:1101/resource/authority/health-activity/OBSERVATIONAL_DATA,http://13.81.34.152:1101/resource/authority/health-activity/SURVEILLANCE</v>
+        <v>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/EHEALTH_APPLICATION,https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/OBSERVATIONAL_DATA,https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/SURVEILLANCE</v>
       </c>
       <c r="H1" t="str">
         <f>IFERROR(INDEX(Health_Activities[Uri], MATCH(Dataset!H65, Health_Activities[Label], 0)),"")</f>
-        <v>http://13.81.34.152:1101/resource/authority/health-activity/EHEALTH_APPLICATION</v>
+        <v>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/EHEALTH_APPLICATION</v>
       </c>
       <c r="I1" t="str">
         <f>IFERROR(INDEX(Health_Activities[Uri], MATCH(Dataset!I65, Health_Activities[Label], 0)),"")</f>
-        <v>http://13.81.34.152:1101/resource/authority/health-activity/OBSERVATIONAL_DATA</v>
+        <v>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/OBSERVATIONAL_DATA</v>
       </c>
       <c r="J1" t="str">
         <f>IFERROR(INDEX(Health_Activities[Uri], MATCH(Dataset!J65, Health_Activities[Label], 0)),"")</f>
-        <v>http://13.81.34.152:1101/resource/authority/health-activity/SURVEILLANCE</v>
+        <v>https://hdeu-dcat.acceptance.data.health.europa.eu/resource/authority/health-activity/SURVEILLANCE</v>
       </c>
       <c r="K1" t="str">
         <f>IFERROR(INDEX(Health_Activities[Uri], MATCH(Dataset!K65, Health_Activities[Label], 0)), "")</f>

</xml_diff>